<commit_message>
Enhance search functionality and data handling in app.js
- Integrated search view initialization and refresh logic into app.js, improving user experience when switching to the search view.
- Added global exposure for search view functions to facilitate interaction from other scripts.
- Updated hierarchy-data.json and search-index.json to include additional use cases, enhancing data richness and consistency.
- Refactored loading logic to utilize embedded data instead of fetching, optimizing performance and reducing load times.
</commit_message>
<xml_diff>
--- a/SCE AMI - Process Hierarchy.xlsx
+++ b/SCE AMI - Process Hierarchy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eyus-my.sharepoint.com/personal/tony_calabro_ey_com/Documents/Desktop/Cursor/Hierarchy 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{A154DD94-45E9-4F63-B76F-0ABDCC218A26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E38A6D7-ADCA-4E3B-95EB-09DDB1F5E43A}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{A154DD94-45E9-4F63-B76F-0ABDCC218A26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A88DAD2B-E7B4-4513-96A9-32A5250D9FEE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C5CF7D8D-18C1-4DA6-BBC5-CBC3C1BDFBAD}"/>
   </bookViews>
@@ -1062,10 +1062,6 @@
     <t>Process and analyze high-volume stream of device events (e.g., power fail, restore, tamper, diagnostic flags) flowing from the HES into the MDMS or event correlation engine, filtering noise to identify actionable conditions for grid operations, revenue protection, or asset management.</t>
   </si>
   <si>
-    <t>Use Case 13 – Post Event Analysis
-Use Case 5 – Advanced Outage Identification and Location Awareness</t>
-  </si>
-  <si>
     <t>Release 1 handles basic alarms. Release 3 (Post Event Analysis) requires correlating these events with SCADA/OMS data for complex root cause analysis.</t>
   </si>
   <si>
@@ -2543,6 +2539,11 @@
   </si>
   <si>
     <t>Use Case 8 – Anomaly &amp; Fault Detection BTM</t>
+  </si>
+  <si>
+    <t>Use Case 13 – Post Event Analysis
+Use Case 5 – Advanced Outage Identification and Location Awareness
+Use Case 9 - Environmental Monitoring</t>
   </si>
 </sst>
 </file>
@@ -4405,7 +4406,7 @@
       <c r="J2" s="10"/>
       <c r="K2" s="10"/>
       <c r="L2" s="10" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4437,7 +4438,7 @@
       <c r="J3" s="10"/>
       <c r="K3" s="10"/>
       <c r="L3" s="10" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4469,7 +4470,7 @@
       <c r="J4" s="10"/>
       <c r="K4" s="10"/>
       <c r="L4" s="10" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
@@ -6800,7 +6801,7 @@
         <v>250</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="F82" s="10" t="s">
         <v>72</v>
@@ -7334,13 +7335,13 @@
         <v>309</v>
       </c>
       <c r="E100" s="10" t="s">
-        <v>310</v>
+        <v>712</v>
       </c>
       <c r="F100" s="10" t="s">
         <v>184</v>
       </c>
       <c r="G100" s="10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H100" s="10" t="s">
         <v>19</v>
@@ -7355,13 +7356,13 @@
         <v>298</v>
       </c>
       <c r="B101" s="10" t="s">
+        <v>311</v>
+      </c>
+      <c r="C101" s="10" t="s">
         <v>312</v>
       </c>
-      <c r="C101" s="10" t="s">
+      <c r="D101" s="10" t="s">
         <v>313</v>
-      </c>
-      <c r="D101" s="10" t="s">
-        <v>314</v>
       </c>
       <c r="E101" s="10" t="s">
         <v>16</v>
@@ -7370,7 +7371,7 @@
         <v>302</v>
       </c>
       <c r="G101" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H101" s="10" t="s">
         <v>19</v>
@@ -7385,22 +7386,22 @@
         <v>298</v>
       </c>
       <c r="B102" s="10" t="s">
+        <v>315</v>
+      </c>
+      <c r="C102" s="10" t="s">
         <v>316</v>
       </c>
-      <c r="C102" s="10" t="s">
+      <c r="D102" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="D102" s="12" t="s">
+      <c r="E102" s="10" t="s">
         <v>318</v>
-      </c>
-      <c r="E102" s="10" t="s">
-        <v>319</v>
       </c>
       <c r="F102" s="10" t="s">
         <v>72</v>
       </c>
       <c r="G102" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H102" s="10" t="s">
         <v>19</v>
@@ -7415,13 +7416,13 @@
         <v>298</v>
       </c>
       <c r="B103" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="C103" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="C103" s="10" t="s">
+      <c r="D103" s="10" t="s">
         <v>322</v>
-      </c>
-      <c r="D103" s="10" t="s">
-        <v>323</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>194</v>
@@ -7448,13 +7449,13 @@
         <v>307</v>
       </c>
       <c r="C104" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="D104" s="12" t="s">
         <v>324</v>
       </c>
-      <c r="D104" s="12" t="s">
+      <c r="E104" s="10" t="s">
         <v>325</v>
-      </c>
-      <c r="E104" s="10" t="s">
-        <v>326</v>
       </c>
       <c r="F104" s="10" t="s">
         <v>131</v>
@@ -7475,16 +7476,16 @@
         <v>298</v>
       </c>
       <c r="B105" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="C105" s="10" t="s">
         <v>327</v>
       </c>
-      <c r="C105" s="10" t="s">
+      <c r="D105" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="D105" s="10" t="s">
+      <c r="E105" s="10" t="s">
         <v>329</v>
-      </c>
-      <c r="E105" s="10" t="s">
-        <v>330</v>
       </c>
       <c r="F105" s="10" t="s">
         <v>131</v>
@@ -7505,13 +7506,13 @@
         <v>298</v>
       </c>
       <c r="B106" s="10" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C106" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="D106" s="10" t="s">
         <v>331</v>
-      </c>
-      <c r="D106" s="10" t="s">
-        <v>332</v>
       </c>
       <c r="E106" s="10" t="s">
         <v>278</v>
@@ -7538,13 +7539,13 @@
         <v>307</v>
       </c>
       <c r="C107" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="D107" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="D107" s="12" t="s">
+      <c r="E107" s="10" t="s">
         <v>334</v>
-      </c>
-      <c r="E107" s="10" t="s">
-        <v>335</v>
       </c>
       <c r="F107" s="10" t="s">
         <v>131</v>
@@ -7719,18 +7720,18 @@
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="P1" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="Q1" s="9" t="s">
         <v>336</v>
-      </c>
-      <c r="Q1" s="9" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="O2" s="13" t="s">
+        <v>337</v>
+      </c>
+      <c r="P2" s="15" t="s">
         <v>338</v>
-      </c>
-      <c r="P2" s="15" t="s">
-        <v>339</v>
       </c>
       <c r="Q2" s="15">
         <v>0</v>
@@ -7738,66 +7739,66 @@
     </row>
     <row r="3" spans="1:17" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="O3" s="14" t="s">
+        <v>339</v>
+      </c>
+      <c r="P3" s="16" t="s">
         <v>340</v>
       </c>
-      <c r="P3" s="16" t="s">
-        <v>341</v>
-      </c>
       <c r="Q3" s="16" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="O4" s="14" t="s">
+        <v>341</v>
+      </c>
+      <c r="P4" s="16" t="s">
         <v>342</v>
       </c>
-      <c r="P4" s="16" t="s">
+      <c r="Q4" s="16" t="s">
         <v>343</v>
-      </c>
-      <c r="Q4" s="16" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="O5" s="14" t="s">
+        <v>344</v>
+      </c>
+      <c r="P5" s="16" t="s">
         <v>345</v>
       </c>
-      <c r="P5" s="16" t="s">
+      <c r="Q5" s="16" t="s">
         <v>346</v>
-      </c>
-      <c r="Q5" s="16" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="E6" t="s">
         <v>348</v>
       </c>
-      <c r="E6" t="s">
-        <v>349</v>
-      </c>
       <c r="I6" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>336</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>337</v>
-      </c>
       <c r="F7" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>336</v>
       </c>
-      <c r="G7" s="9" t="s">
-        <v>337</v>
-      </c>
       <c r="J7" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="K7" s="9" t="s">
         <v>336</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -7898,10 +7899,10 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="B18" t="s">
         <v>350</v>
-      </c>
-      <c r="B18" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -7962,7 +7963,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B26">
         <v>106</v>
@@ -8002,13 +8003,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>354</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -8019,10 +8020,10 @@
         <v>26</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>356</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>357</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>25</v>
@@ -8037,7 +8038,7 @@
         <v>19</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -8048,10 +8049,10 @@
         <v>180</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>359</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>360</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>183</v>
@@ -8060,10 +8061,10 @@
         <v>38</v>
       </c>
       <c r="G3" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>361</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>362</v>
       </c>
       <c r="I3" s="4"/>
     </row>
@@ -8075,10 +8076,10 @@
         <v>172</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>363</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>364</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>52</v>
@@ -8087,72 +8088,72 @@
         <v>131</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I4" s="4"/>
     </row>
     <row r="5" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>367</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>369</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>370</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I5" s="4"/>
     </row>
     <row r="6" spans="1:9" ht="195" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>367</v>
-      </c>
       <c r="C6" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>373</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>53</v>
@@ -8161,36 +8162,36 @@
         <v>87</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="I7" s="4" t="s">
         <v>376</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>362</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>379</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>380</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>25</v>
@@ -8199,118 +8200,118 @@
         <v>17</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I8" s="4"/>
     </row>
     <row r="9" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>49</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>382</v>
-      </c>
       <c r="E9" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I9" s="4"/>
     </row>
     <row r="10" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>385</v>
-      </c>
       <c r="E10" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I10" s="4"/>
     </row>
     <row r="11" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>387</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I11" s="4"/>
     </row>
     <row r="12" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>390</v>
-      </c>
       <c r="E12" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I12" s="4"/>
     </row>
@@ -8319,170 +8320,170 @@
         <v>298</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>393</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>38</v>
       </c>
       <c r="G13" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>394</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>362</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="195" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>397</v>
-      </c>
       <c r="E14" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G14" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="I14" s="4" t="s">
         <v>398</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>362</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C15" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>401</v>
-      </c>
       <c r="E15" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>17</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C16" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>403</v>
-      </c>
       <c r="E16" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="195" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C17" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>406</v>
-      </c>
       <c r="E17" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G17" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="I17" s="4" t="s">
         <v>398</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>362</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="195" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C18" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>408</v>
-      </c>
       <c r="E18" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G18" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="I18" s="4" t="s">
         <v>398</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>362</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="60" x14ac:dyDescent="0.25">
@@ -8493,42 +8494,42 @@
         <v>121</v>
       </c>
       <c r="C19" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>410</v>
-      </c>
       <c r="E19" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>413</v>
-      </c>
       <c r="E20" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>38</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
@@ -8539,10 +8540,10 @@
         <v>180</v>
       </c>
       <c r="C21" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>415</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>416</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>183</v>
@@ -8554,13 +8555,13 @@
         <v>22</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="I21" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="J21" s="4" t="s">
         <v>417</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="75" x14ac:dyDescent="0.25">
@@ -8571,13 +8572,13 @@
         <v>172</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>420</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>421</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>175</v>
@@ -8594,10 +8595,10 @@
         <v>172</v>
       </c>
       <c r="C23" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>422</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>423</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>52</v>
@@ -8614,13 +8615,13 @@
         <v>120</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>424</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="D24" s="2" t="s">
         <v>425</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>426</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>183</v>
@@ -8632,13 +8633,13 @@
         <v>19</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="I24" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="J24" s="4" t="s">
         <v>427</v>
-      </c>
-      <c r="J24" s="4" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="60" x14ac:dyDescent="0.25">
@@ -8646,16 +8647,16 @@
         <v>42</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C25" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>430</v>
-      </c>
       <c r="E25" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>17</v>
@@ -8669,13 +8670,13 @@
         <v>42</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="D26" s="2" t="s">
         <v>432</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>433</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>25</v>
@@ -8687,7 +8688,7 @@
         <v>46</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
@@ -8697,13 +8698,13 @@
         <v>195</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="D27" s="2" t="s">
         <v>436</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>437</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>258</v>
@@ -8720,13 +8721,13 @@
         <v>195</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C28" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>438</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>439</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>258</v>
@@ -8743,13 +8744,13 @@
         <v>298</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>440</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="D29" s="2" t="s">
         <v>441</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>442</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>25</v>
@@ -8761,13 +8762,13 @@
         <v>46</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I29" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="J29" s="2" t="s">
         <v>443</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="300" x14ac:dyDescent="0.25">
@@ -8775,13 +8776,13 @@
         <v>298</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C30" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>445</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>446</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>25</v>
@@ -8793,13 +8794,13 @@
         <v>19</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I30" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="J30" s="2" t="s">
         <v>447</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="195" x14ac:dyDescent="0.25">
@@ -8807,13 +8808,13 @@
         <v>298</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C31" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>449</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>450</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>25</v>
@@ -8825,13 +8826,13 @@
         <v>19</v>
       </c>
       <c r="H31" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="I31" s="4" t="s">
         <v>451</v>
       </c>
-      <c r="I31" s="4" t="s">
+      <c r="J31" s="2" t="s">
         <v>452</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="255" x14ac:dyDescent="0.25">
@@ -8839,16 +8840,16 @@
         <v>298</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C32" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>454</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>455</v>
-      </c>
       <c r="E32" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>72</v>
@@ -8857,13 +8858,13 @@
         <v>19</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I32" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="J32" s="2" t="s">
         <v>456</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="240" x14ac:dyDescent="0.25">
@@ -8871,16 +8872,16 @@
         <v>298</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C33" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>459</v>
-      </c>
       <c r="E33" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>72</v>
@@ -8889,13 +8890,13 @@
         <v>19</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I33" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="J33" s="2" t="s">
         <v>460</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="150" x14ac:dyDescent="0.25">
@@ -8903,16 +8904,16 @@
         <v>298</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C34" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>463</v>
-      </c>
       <c r="E34" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>38</v>
@@ -8921,13 +8922,13 @@
         <v>19</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I34" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="J34" s="2" t="s">
         <v>464</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="165" x14ac:dyDescent="0.25">
@@ -8935,16 +8936,16 @@
         <v>298</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C35" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="D35" s="2" t="s">
-        <v>467</v>
-      </c>
       <c r="E35" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>131</v>
@@ -8953,13 +8954,13 @@
         <v>19</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I35" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="J35" s="2" t="s">
         <v>468</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="150" x14ac:dyDescent="0.25">
@@ -8967,16 +8968,16 @@
         <v>298</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="C36" s="3" t="s">
         <v>470</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="D36" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="E36" s="2" t="s">
         <v>472</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>473</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>38</v>
@@ -8985,13 +8986,13 @@
         <v>46</v>
       </c>
       <c r="H36" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="I36" s="4" t="s">
         <v>474</v>
       </c>
-      <c r="I36" s="4" t="s">
+      <c r="J36" s="2" t="s">
         <v>475</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="45" x14ac:dyDescent="0.25">
@@ -8999,16 +9000,16 @@
         <v>298</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C37" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>477</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="E37" s="2" t="s">
         <v>478</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>479</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>131</v>
@@ -9022,16 +9023,16 @@
         <v>298</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C38" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>481</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>482</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>131</v>
@@ -9045,16 +9046,16 @@
         <v>298</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C39" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>483</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="E39" s="2" t="s">
         <v>484</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>485</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>131</v>
@@ -9071,13 +9072,13 @@
         <v>299</v>
       </c>
       <c r="C40" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>486</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>487</v>
-      </c>
       <c r="E40" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>72</v>
@@ -9086,13 +9087,13 @@
         <v>19</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I40" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="J40" s="2" t="s">
         <v>488</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>489</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="60" x14ac:dyDescent="0.25">
@@ -9103,13 +9104,13 @@
         <v>299</v>
       </c>
       <c r="C41" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>490</v>
       </c>
-      <c r="D41" s="2" t="s">
-        <v>491</v>
-      </c>
       <c r="E41" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>38</v>
@@ -9123,16 +9124,16 @@
         <v>298</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="C42" s="3" t="s">
         <v>492</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="D42" s="2" t="s">
         <v>493</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>494</v>
-      </c>
       <c r="E42" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>38</v>
@@ -9146,16 +9147,16 @@
         <v>298</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C43" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>495</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>496</v>
-      </c>
       <c r="E43" s="2" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>131</v>
@@ -9169,16 +9170,16 @@
         <v>298</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C44" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>497</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>498</v>
-      </c>
       <c r="E44" s="2" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>131</v>
@@ -9192,16 +9193,16 @@
         <v>298</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C45" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>500</v>
-      </c>
       <c r="E45" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>131</v>
@@ -9265,10 +9266,10 @@
         <v>13</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>501</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>502</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>16</v>
@@ -9291,10 +9292,10 @@
         <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>503</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>504</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>16</v>
@@ -9317,10 +9318,10 @@
         <v>13</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>505</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>506</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>16</v>
@@ -9346,7 +9347,7 @@
         <v>20</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>16</v>
@@ -9372,7 +9373,7 @@
         <v>23</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>25</v>
@@ -9398,7 +9399,7 @@
         <v>36</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>16</v>
@@ -9421,10 +9422,10 @@
         <v>31</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>510</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>511</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>16</v>
@@ -9450,7 +9451,7 @@
         <v>27</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>16</v>
@@ -9476,7 +9477,7 @@
         <v>29</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>16</v>
@@ -9499,10 +9500,10 @@
         <v>43</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>514</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>515</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>16</v>
@@ -9525,10 +9526,10 @@
         <v>43</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>516</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>517</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>16</v>
@@ -9554,7 +9555,7 @@
         <v>50</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>52</v>
@@ -9577,10 +9578,10 @@
         <v>53</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>519</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>520</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>16</v>
@@ -9606,7 +9607,7 @@
         <v>58</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>16</v>
@@ -9632,7 +9633,7 @@
         <v>67</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>16</v>
@@ -9658,7 +9659,7 @@
         <v>60</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>52</v>
@@ -9681,10 +9682,10 @@
         <v>62</v>
       </c>
       <c r="C18" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>524</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>525</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>16</v>
@@ -9710,7 +9711,7 @@
         <v>47</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>16</v>
@@ -9733,19 +9734,19 @@
         <v>104</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>527</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>528</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>529</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>72</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>19</v>
@@ -9759,19 +9760,19 @@
         <v>104</v>
       </c>
       <c r="C21" s="3" t="s">
+        <v>530</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>531</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>532</v>
-      </c>
       <c r="E21" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>72</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>19</v>
@@ -9785,10 +9786,10 @@
         <v>104</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>534</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>535</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>25</v>
@@ -9811,10 +9812,10 @@
         <v>104</v>
       </c>
       <c r="C23" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>536</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>537</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>111</v>
@@ -9837,10 +9838,10 @@
         <v>104</v>
       </c>
       <c r="C24" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>538</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>539</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>111</v>
@@ -9849,7 +9850,7 @@
         <v>72</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>22</v>
@@ -9866,7 +9867,7 @@
         <v>117</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>86</v>
@@ -9889,10 +9890,10 @@
         <v>121</v>
       </c>
       <c r="C26" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>542</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>543</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>111</v>
@@ -9918,10 +9919,10 @@
         <v>145</v>
       </c>
       <c r="D27" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>544</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>545</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>17</v>
@@ -9944,10 +9945,10 @@
         <v>148</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>17</v>
@@ -9970,7 +9971,7 @@
         <v>134</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>111</v>
@@ -9993,10 +9994,10 @@
         <v>121</v>
       </c>
       <c r="C30" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>548</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>549</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>111</v>
@@ -10022,7 +10023,7 @@
         <v>142</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>111</v>
@@ -10045,10 +10046,10 @@
         <v>180</v>
       </c>
       <c r="C32" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>551</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>552</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>183</v>
@@ -10071,10 +10072,10 @@
         <v>180</v>
       </c>
       <c r="C33" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>553</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>554</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>183</v>
@@ -10083,7 +10084,7 @@
         <v>184</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>19</v>
@@ -10100,10 +10101,10 @@
         <v>186</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>556</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>557</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>131</v>
@@ -10126,10 +10127,10 @@
         <v>188</v>
       </c>
       <c r="D35" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>558</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>559</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>131</v>
@@ -10149,10 +10150,10 @@
         <v>155</v>
       </c>
       <c r="C36" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>560</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>561</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>86</v>
@@ -10175,10 +10176,10 @@
         <v>155</v>
       </c>
       <c r="C37" s="3" t="s">
+        <v>561</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>562</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>563</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>86</v>
@@ -10201,10 +10202,10 @@
         <v>155</v>
       </c>
       <c r="C38" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>564</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>565</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>86</v>
@@ -10230,7 +10231,7 @@
         <v>173</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>52</v>
@@ -10253,10 +10254,10 @@
         <v>150</v>
       </c>
       <c r="C40" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>567</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>568</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>52</v>
@@ -10279,10 +10280,10 @@
         <v>150</v>
       </c>
       <c r="C41" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>569</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>570</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>52</v>
@@ -10308,7 +10309,7 @@
         <v>122</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>124</v>
@@ -10331,10 +10332,10 @@
         <v>191</v>
       </c>
       <c r="C43" s="3" t="s">
+        <v>571</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>572</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>573</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>194</v>
@@ -10357,10 +10358,10 @@
         <v>191</v>
       </c>
       <c r="C44" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>574</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>575</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>194</v>
@@ -10383,10 +10384,10 @@
         <v>191</v>
       </c>
       <c r="C45" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>576</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>577</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>194</v>
@@ -10409,10 +10410,10 @@
         <v>177</v>
       </c>
       <c r="C46" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>578</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>579</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>16</v>
@@ -10435,10 +10436,10 @@
         <v>177</v>
       </c>
       <c r="C47" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>580</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>581</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>16</v>
@@ -10464,7 +10465,7 @@
         <v>160</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>16</v>
@@ -10490,7 +10491,7 @@
         <v>162</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>16</v>
@@ -10516,7 +10517,7 @@
         <v>164</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>16</v>
@@ -10542,7 +10543,7 @@
         <v>166</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>16</v>
@@ -10565,10 +10566,10 @@
         <v>159</v>
       </c>
       <c r="C52" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>586</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>587</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>16</v>
@@ -10594,7 +10595,7 @@
         <v>70</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>25</v>
@@ -10620,7 +10621,7 @@
         <v>74</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>25</v>
@@ -10646,7 +10647,7 @@
         <v>99</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>25</v>
@@ -10672,7 +10673,7 @@
         <v>101</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>16</v>
@@ -10695,10 +10696,10 @@
         <v>53</v>
       </c>
       <c r="C57" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>592</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>593</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>16</v>
@@ -10707,7 +10708,7 @@
         <v>72</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>19</v>
@@ -10724,7 +10725,7 @@
         <v>77</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>16</v>
@@ -10747,10 +10748,10 @@
         <v>76</v>
       </c>
       <c r="C59" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>596</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>597</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>16</v>
@@ -10759,7 +10760,7 @@
         <v>72</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>19</v>
@@ -10776,7 +10777,7 @@
         <v>87</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>16</v>
@@ -10799,13 +10800,13 @@
         <v>76</v>
       </c>
       <c r="C61" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="D61" s="2" t="s">
         <v>599</v>
       </c>
-      <c r="D61" s="2" t="s">
+      <c r="E61" s="2" t="s">
         <v>600</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>601</v>
       </c>
       <c r="F61" s="2" t="s">
         <v>17</v>
@@ -10822,13 +10823,13 @@
         <v>69</v>
       </c>
       <c r="B62" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="C62" s="3" t="s">
         <v>602</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="D62" s="2" t="s">
         <v>603</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>604</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>16</v>
@@ -10854,7 +10855,7 @@
         <v>94</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>16</v>
@@ -10880,7 +10881,7 @@
         <v>96</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>16</v>
@@ -10903,10 +10904,10 @@
         <v>89</v>
       </c>
       <c r="C65" s="3" t="s">
+        <v>606</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>607</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>608</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>16</v>
@@ -10929,10 +10930,10 @@
         <v>255</v>
       </c>
       <c r="C66" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>609</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>610</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>258</v>
@@ -10955,10 +10956,10 @@
         <v>255</v>
       </c>
       <c r="C67" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="D67" s="2" t="s">
         <v>611</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>612</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>258</v>
@@ -10981,10 +10982,10 @@
         <v>255</v>
       </c>
       <c r="C68" s="3" t="s">
+        <v>612</v>
+      </c>
+      <c r="D68" s="2" t="s">
         <v>613</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>614</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>258</v>
@@ -11007,10 +11008,10 @@
         <v>255</v>
       </c>
       <c r="C69" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="D69" s="2" t="s">
         <v>615</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>616</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>258</v>
@@ -11019,7 +11020,7 @@
         <v>175</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="H69" s="2" t="s">
         <v>19</v>
@@ -11036,16 +11037,16 @@
         <v>267</v>
       </c>
       <c r="D70" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="E70" s="2" t="s">
         <v>618</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>619</v>
       </c>
       <c r="F70" s="2" t="s">
         <v>175</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>19</v>
@@ -11056,13 +11057,13 @@
         <v>195</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C71" s="3" t="s">
         <v>262</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>258</v>
@@ -11088,7 +11089,7 @@
         <v>223</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>83</v>
@@ -11097,7 +11098,7 @@
         <v>72</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>46</v>
@@ -11111,10 +11112,10 @@
         <v>222</v>
       </c>
       <c r="C73" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>624</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>625</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>228</v>
@@ -11137,10 +11138,10 @@
         <v>261</v>
       </c>
       <c r="C74" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="D74" s="2" t="s">
         <v>626</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>627</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>228</v>
@@ -11163,10 +11164,10 @@
         <v>261</v>
       </c>
       <c r="C75" s="3" t="s">
+        <v>627</v>
+      </c>
+      <c r="D75" s="2" t="s">
         <v>628</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>629</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>228</v>
@@ -11192,7 +11193,7 @@
         <v>232</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>83</v>
@@ -11201,7 +11202,7 @@
         <v>72</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="H76" s="2" t="s">
         <v>19</v>
@@ -11218,7 +11219,7 @@
         <v>235</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>83</v>
@@ -11227,7 +11228,7 @@
         <v>72</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="H77" s="2" t="s">
         <v>19</v>
@@ -11241,10 +11242,10 @@
         <v>231</v>
       </c>
       <c r="C78" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="D78" s="2" t="s">
         <v>633</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>634</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>83</v>
@@ -11253,7 +11254,7 @@
         <v>175</v>
       </c>
       <c r="G78" s="4" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="H78" s="2" t="s">
         <v>46</v>
@@ -11270,16 +11271,16 @@
         <v>249</v>
       </c>
       <c r="D79" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="E79" s="2" t="s">
         <v>636</v>
-      </c>
-      <c r="E79" s="2" t="s">
-        <v>637</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>72</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="H79" s="2" t="s">
         <v>19</v>
@@ -11296,10 +11297,10 @@
         <v>252</v>
       </c>
       <c r="D80" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="E80" s="2" t="s">
         <v>639</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>640</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>38</v>
@@ -11322,7 +11323,7 @@
         <v>209</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>211</v>
@@ -11345,10 +11346,10 @@
         <v>208</v>
       </c>
       <c r="C82" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="D82" s="2" t="s">
         <v>642</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>643</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>211</v>
@@ -11374,10 +11375,10 @@
         <v>219</v>
       </c>
       <c r="D83" s="2" t="s">
+        <v>643</v>
+      </c>
+      <c r="E83" s="2" t="s">
         <v>644</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>645</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>38</v>
@@ -11400,10 +11401,10 @@
         <v>216</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="F84" s="2" t="s">
         <v>131</v>
@@ -11423,10 +11424,10 @@
         <v>196</v>
       </c>
       <c r="C85" s="3" t="s">
+        <v>646</v>
+      </c>
+      <c r="D85" s="2" t="s">
         <v>647</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>648</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>203</v>
@@ -11449,10 +11450,10 @@
         <v>196</v>
       </c>
       <c r="C86" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="D86" s="2" t="s">
         <v>649</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>650</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>203</v>
@@ -11461,7 +11462,7 @@
         <v>175</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="H86" s="2" t="s">
         <v>19</v>
@@ -11478,7 +11479,7 @@
         <v>201</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>203</v>
@@ -11501,10 +11502,10 @@
         <v>196</v>
       </c>
       <c r="C88" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="D88" s="2" t="s">
         <v>653</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>654</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>203</v>
@@ -11527,10 +11528,10 @@
         <v>243</v>
       </c>
       <c r="C89" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="D89" s="2" t="s">
         <v>655</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>656</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>246</v>
@@ -11539,7 +11540,7 @@
         <v>175</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="H89" s="2" t="s">
         <v>19</v>
@@ -11553,10 +11554,10 @@
         <v>243</v>
       </c>
       <c r="C90" s="3" t="s">
+        <v>657</v>
+      </c>
+      <c r="D90" s="2" t="s">
         <v>658</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>659</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>246</v>
@@ -11579,19 +11580,19 @@
         <v>243</v>
       </c>
       <c r="C91" s="3" t="s">
+        <v>659</v>
+      </c>
+      <c r="D91" s="2" t="s">
         <v>660</v>
       </c>
-      <c r="D91" s="2" t="s">
+      <c r="E91" s="2" t="s">
         <v>661</v>
-      </c>
-      <c r="E91" s="2" t="s">
-        <v>662</v>
       </c>
       <c r="F91" s="2" t="s">
         <v>175</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="H91" s="2" t="s">
         <v>19</v>
@@ -11608,16 +11609,16 @@
         <v>272</v>
       </c>
       <c r="D92" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="E92" s="2" t="s">
         <v>664</v>
-      </c>
-      <c r="E92" s="2" t="s">
-        <v>665</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>175</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="H92" s="2" t="s">
         <v>46</v>
@@ -11631,10 +11632,10 @@
         <v>271</v>
       </c>
       <c r="C93" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="D93" s="2" t="s">
         <v>667</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>668</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>278</v>
@@ -11657,10 +11658,10 @@
         <v>271</v>
       </c>
       <c r="C94" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="D94" s="2" t="s">
         <v>669</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>670</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>278</v>
@@ -11683,10 +11684,10 @@
         <v>271</v>
       </c>
       <c r="C95" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="D95" s="2" t="s">
         <v>671</v>
-      </c>
-      <c r="D95" s="2" t="s">
-        <v>672</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>278</v>
@@ -11712,7 +11713,7 @@
         <v>205</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>207</v>
@@ -11732,13 +11733,13 @@
         <v>279</v>
       </c>
       <c r="B97" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="C97" s="3" t="s">
         <v>674</v>
       </c>
-      <c r="C97" s="3" t="s">
+      <c r="D97" s="2" t="s">
         <v>675</v>
-      </c>
-      <c r="D97" s="2" t="s">
-        <v>676</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>25</v>
@@ -11758,13 +11759,13 @@
         <v>279</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="C98" s="3" t="s">
+        <v>676</v>
+      </c>
+      <c r="D98" s="2" t="s">
         <v>677</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>678</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>25</v>
@@ -11784,16 +11785,16 @@
         <v>279</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="C99" s="3" t="s">
         <v>283</v>
       </c>
       <c r="D99" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="E99" s="2" t="s">
         <v>680</v>
-      </c>
-      <c r="E99" s="2" t="s">
-        <v>681</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>17</v>
@@ -11816,7 +11817,7 @@
         <v>291</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>16</v>
@@ -11842,7 +11843,7 @@
         <v>293</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>25</v>
@@ -11868,7 +11869,7 @@
         <v>295</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E102" s="2" t="s">
         <v>25</v>
@@ -11888,13 +11889,13 @@
         <v>279</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C103" s="3" t="s">
+        <v>684</v>
+      </c>
+      <c r="D103" s="2" t="s">
         <v>685</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>686</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>25</v>
@@ -11914,13 +11915,13 @@
         <v>279</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C104" s="3" t="s">
+        <v>686</v>
+      </c>
+      <c r="D104" s="2" t="s">
         <v>687</v>
-      </c>
-      <c r="D104" s="2" t="s">
-        <v>688</v>
       </c>
       <c r="E104" s="2" t="s">
         <v>25</v>
@@ -11940,13 +11941,13 @@
         <v>279</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C105" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="D105" s="2" t="s">
         <v>689</v>
-      </c>
-      <c r="D105" s="2" t="s">
-        <v>690</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>25</v>
@@ -11966,13 +11967,13 @@
         <v>298</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C106" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="D106" s="2" t="s">
         <v>691</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>692</v>
       </c>
       <c r="E106" s="2" t="s">
         <v>194</v>
@@ -11992,13 +11993,13 @@
         <v>298</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C107" s="3" t="s">
+        <v>692</v>
+      </c>
+      <c r="D107" s="2" t="s">
         <v>693</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>694</v>
       </c>
       <c r="E107" s="2" t="s">
         <v>194</v>
@@ -12018,13 +12019,13 @@
         <v>298</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E108" s="2" t="s">
         <v>194</v>
@@ -12050,7 +12051,7 @@
         <v>300</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E109" s="2" t="s">
         <v>16</v>
@@ -12073,13 +12074,13 @@
         <v>307</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D110" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="E110" s="2" t="s">
         <v>697</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>698</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>131</v>
@@ -12102,16 +12103,16 @@
         <v>308</v>
       </c>
       <c r="D111" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="E111" s="2" t="s">
         <v>699</v>
-      </c>
-      <c r="E111" s="2" t="s">
-        <v>700</v>
       </c>
       <c r="F111" s="2" t="s">
         <v>184</v>
       </c>
       <c r="G111" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H111" s="2" t="s">
         <v>19</v>
@@ -12122,13 +12123,13 @@
         <v>298</v>
       </c>
       <c r="B112" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="C112" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="C112" s="3" t="s">
-        <v>313</v>
-      </c>
       <c r="D112" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>16</v>
@@ -12137,7 +12138,7 @@
         <v>302</v>
       </c>
       <c r="G112" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H112" s="2" t="s">
         <v>19</v>
@@ -12148,22 +12149,22 @@
         <v>298</v>
       </c>
       <c r="B113" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C113" s="3" t="s">
         <v>316</v>
       </c>
-      <c r="C113" s="3" t="s">
-        <v>317</v>
-      </c>
       <c r="D113" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="E113" s="2" t="s">
         <v>702</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>703</v>
       </c>
       <c r="F113" s="2" t="s">
         <v>72</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H113" s="2" t="s">
         <v>19</v>
@@ -12174,16 +12175,16 @@
         <v>298</v>
       </c>
       <c r="B114" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C114" s="3" t="s">
         <v>327</v>
       </c>
-      <c r="C114" s="3" t="s">
-        <v>328</v>
-      </c>
       <c r="D114" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="E114" s="2" t="s">
         <v>704</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>705</v>
       </c>
       <c r="F114" s="2" t="s">
         <v>131</v>
@@ -12200,13 +12201,13 @@
         <v>298</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E115" s="2" t="s">
         <v>278</v>
@@ -12229,13 +12230,13 @@
         <v>307</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D116" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="E116" s="2" t="s">
         <v>707</v>
-      </c>
-      <c r="E116" s="2" t="s">
-        <v>708</v>
       </c>
       <c r="F116" s="2" t="s">
         <v>131</v>
@@ -12264,6 +12265,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="139fca70-673f-44e1-94c2-b523bb9c108c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="7eaf932d-7370-48c5-9459-ae540daf9d7d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DFB9E5947890A84F90C1025035B3A9E9" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="abb99fc9a48c7a251434465201697796">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="139fca70-673f-44e1-94c2-b523bb9c108c" xmlns:ns3="7eaf932d-7370-48c5-9459-ae540daf9d7d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d5c101f0e739d89bf88b83005715ab8d" ns2:_="" ns3:_="">
     <xsd:import namespace="139fca70-673f-44e1-94c2-b523bb9c108c"/>
@@ -12470,17 +12482,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="139fca70-673f-44e1-94c2-b523bb9c108c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="7eaf932d-7370-48c5-9459-ae540daf9d7d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3BB2BB8B-BA4E-4835-AC34-431A62162A7D}">
   <ds:schemaRefs>
@@ -12490,6 +12491,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B57CF69-5D19-450C-935B-68EC43A8DA31}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="139fca70-673f-44e1-94c2-b523bb9c108c"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="7eaf932d-7370-48c5-9459-ae540daf9d7d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82D5B6C7-9BF1-46B8-8CAF-B305B78CEC57}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12506,21 +12524,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B57CF69-5D19-450C-935B-68EC43A8DA31}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="139fca70-673f-44e1-94c2-b523bb9c108c"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="7eaf932d-7370-48c5-9459-ae540daf9d7d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update hierarchy and search data for improved process management
- Removed the "Calculate and validate register-based bills" entry from hierarchy-data.json, search-index.json, and standalone.html to streamline the process hierarchy.
- Renamed "Manage Virtual Net Metering (VNM) Allocations" and "Manage NEM Aggregation (NEM-A) Structures" to "Manage Program-Based Virtual Net Metering (VNM) Allocations" and "Manage Program-Based NEM Aggregation Structures" respectively for clarity.
- Added a new entry for "Manage Platform-Based Complex Metering Relationships" to enhance the hierarchy with additional process details.
- Updated use cases and IT release versions for several processes to ensure consistency across the application.
</commit_message>
<xml_diff>
--- a/SCE AMI - Process Hierarchy.xlsx
+++ b/SCE AMI - Process Hierarchy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eyus-my.sharepoint.com/personal/tony_calabro_ey_com/Documents/Desktop/Cursor/Hierarchy 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{A154DD94-45E9-4F63-B76F-0ABDCC218A26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A88DAD2B-E7B4-4513-96A9-32A5250D9FEE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{19EDBEB5-A37C-4793-9C0A-C5192023A9DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C5CF7D8D-18C1-4DA6-BBC5-CBC3C1BDFBAD}"/>
   </bookViews>
@@ -118,7 +118,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2207" uniqueCount="713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2218" uniqueCount="720">
   <si>
     <t>L1 Process Name</t>
   </si>
@@ -2544,6 +2544,27 @@
     <t>Use Case 13 – Post Event Analysis
 Use Case 5 – Advanced Outage Identification and Location Awareness
 Use Case 9 - Environmental Monitoring</t>
+  </si>
+  <si>
+    <t>Removed on 1/16, SCE does not do MRO</t>
+  </si>
+  <si>
+    <t>Moved to IT Release 1 per 1/16 meeting. Offered today</t>
+  </si>
+  <si>
+    <t>Moved to IT Release 1 on 1/16.  Part of billing process</t>
+  </si>
+  <si>
+    <t>Manage Program-Based Virtual Net Metering (VNM) Allocations</t>
+  </si>
+  <si>
+    <t>Manage Program-Based NEM Aggregation Structures</t>
+  </si>
+  <si>
+    <t>Manage Platform-Based Complex Metering Relationships</t>
+  </si>
+  <si>
+    <t>Define, configure, and maintain complex metering relationships—including deduct meters, totalizer arrangements, and sub-metering structures—by establishing parent-child device hierarchies, applying aggregation or subtraction rules to interval and register data, and producing auditable billing determinants for accurate CIS settlement.</t>
   </si>
 </sst>
 </file>
@@ -2784,10 +2805,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
-<namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14"/>
-</file>
-
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="Tony Calabro" id="{E164CD4D-F60A-4122-8809-9E91BD6DDA59}" userId="S::Tony.Calabro@ey.com::1559027e-7fee-4795-b2ff-4998584920b1" providerId="AD"/>
@@ -2797,7 +2814,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Tony Calabro" refreshedDate="45992.533690162039" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="106" xr:uid="{DCE9D4D1-60AF-4CA9-896D-C7FDA77BEEFA}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:H107" sheet="Process Hierarchy"/>
+    <worksheetSource ref="A45:H45" sheet="Process Hierarchy"/>
   </cacheSource>
   <cacheFields count="8">
     <cacheField name="L1 Process Name" numFmtId="0">
@@ -4322,7 +4339,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8892926-E8FC-4E51-8265-E6D97D7EE353}">
-  <dimension ref="A1:L140"/>
+  <dimension ref="A1:M140"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" customWidth="1"/>
@@ -4505,7 +4522,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="84" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="91.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>12</v>
       </c>
@@ -5497,7 +5514,7 @@
       <c r="K38" s="10"/>
       <c r="L38" s="10"/>
     </row>
-    <row r="39" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="10" t="s">
         <v>120</v>
       </c>
@@ -5505,10 +5522,10 @@
         <v>121</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="D39" s="17" t="s">
-        <v>133</v>
+        <v>125</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>126</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>111</v>
@@ -5520,7 +5537,7 @@
         <v>18</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="I39" s="10"/>
       <c r="J39" s="10"/>
@@ -5535,10 +5552,10 @@
         <v>121</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E40" s="10" t="s">
         <v>111</v>
@@ -5565,16 +5582,16 @@
         <v>121</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>111</v>
       </c>
       <c r="F41" s="10" t="s">
-        <v>17</v>
+        <v>131</v>
       </c>
       <c r="G41" s="10" t="s">
         <v>18</v>
@@ -5587,7 +5604,7 @@
       <c r="K41" s="10"/>
       <c r="L41" s="10"/>
     </row>
-    <row r="42" spans="1:12" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="10" t="s">
         <v>120</v>
       </c>
@@ -5595,29 +5612,29 @@
         <v>121</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>131</v>
+        <v>17</v>
       </c>
       <c r="G42" s="10" t="s">
         <v>18</v>
       </c>
       <c r="H42" s="10" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="I42" s="10"/>
       <c r="J42" s="10"/>
       <c r="K42" s="10"/>
       <c r="L42" s="10"/>
     </row>
-    <row r="43" spans="1:12" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="10" t="s">
         <v>120</v>
       </c>
@@ -5625,13 +5642,13 @@
         <v>121</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>123</v>
+        <v>134</v>
+      </c>
+      <c r="D43" s="17" t="s">
+        <v>135</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>17</v>
@@ -5640,14 +5657,14 @@
         <v>18</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I43" s="10"/>
       <c r="J43" s="10"/>
       <c r="K43" s="10"/>
       <c r="L43" s="10"/>
     </row>
-    <row r="44" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="10" t="s">
         <v>120</v>
       </c>
@@ -5655,10 +5672,10 @@
         <v>121</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="D44" s="17" t="s">
-        <v>135</v>
+        <v>136</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>137</v>
       </c>
       <c r="E44" s="10" t="s">
         <v>111</v>
@@ -5670,7 +5687,7 @@
         <v>18</v>
       </c>
       <c r="H44" s="10" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="I44" s="10"/>
       <c r="J44" s="10"/>
@@ -5685,16 +5702,16 @@
         <v>121</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>111</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G45" s="10" t="s">
         <v>18</v>
@@ -5707,7 +5724,7 @@
       <c r="K45" s="10"/>
       <c r="L45" s="10"/>
     </row>
-    <row r="46" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" ht="90.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="10" t="s">
         <v>120</v>
       </c>
@@ -5715,16 +5732,16 @@
         <v>121</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E46" s="10" t="s">
         <v>111</v>
       </c>
       <c r="F46" s="10" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="G46" s="10" t="s">
         <v>18</v>
@@ -5737,7 +5754,7 @@
       <c r="K46" s="10"/>
       <c r="L46" s="10"/>
     </row>
-    <row r="47" spans="1:12" ht="90.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="10" t="s">
         <v>120</v>
       </c>
@@ -5745,10 +5762,10 @@
         <v>121</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="D47" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
+      </c>
+      <c r="D47" s="17" t="s">
+        <v>143</v>
       </c>
       <c r="E47" s="10" t="s">
         <v>111</v>
@@ -5760,28 +5777,28 @@
         <v>18</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I47" s="10"/>
       <c r="J47" s="10"/>
       <c r="K47" s="10"/>
       <c r="L47" s="10"/>
     </row>
-    <row r="48" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" ht="78.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="10" t="s">
         <v>120</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="D48" s="17" t="s">
-        <v>143</v>
+        <v>716</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>146</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>111</v>
+        <v>147</v>
       </c>
       <c r="F48" s="10" t="s">
         <v>17</v>
@@ -5790,14 +5807,14 @@
         <v>18</v>
       </c>
       <c r="H48" s="10" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="I48" s="10"/>
       <c r="J48" s="10"/>
       <c r="K48" s="10"/>
       <c r="L48" s="10"/>
     </row>
-    <row r="49" spans="1:12" ht="78.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" ht="94.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="10" t="s">
         <v>120</v>
       </c>
@@ -5805,10 +5822,10 @@
         <v>144</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>145</v>
+        <v>717</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E49" s="10" t="s">
         <v>147</v>
@@ -5827,7 +5844,7 @@
       <c r="K49" s="10"/>
       <c r="L49" s="10"/>
     </row>
-    <row r="50" spans="1:12" ht="94.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" ht="94.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="10" t="s">
         <v>120</v>
       </c>
@@ -5835,13 +5852,13 @@
         <v>144</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>148</v>
+        <v>718</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>149</v>
+        <v>719</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>147</v>
+        <v>111</v>
       </c>
       <c r="F50" s="10" t="s">
         <v>17</v>
@@ -5857,7 +5874,7 @@
       <c r="K50" s="10"/>
       <c r="L50" s="10"/>
     </row>
-    <row r="51" spans="1:12" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="10" t="s">
         <v>120</v>
       </c>
@@ -5887,7 +5904,7 @@
       <c r="K51" s="10"/>
       <c r="L51" s="10"/>
     </row>
-    <row r="52" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10" t="s">
         <v>120</v>
       </c>
@@ -5917,7 +5934,7 @@
       <c r="K52" s="10"/>
       <c r="L52" s="10"/>
     </row>
-    <row r="53" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="10" t="s">
         <v>120</v>
       </c>
@@ -5947,7 +5964,7 @@
       <c r="K53" s="10"/>
       <c r="L53" s="10"/>
     </row>
-    <row r="54" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="10" t="s">
         <v>120</v>
       </c>
@@ -5977,7 +5994,7 @@
       <c r="K54" s="10"/>
       <c r="L54" s="10"/>
     </row>
-    <row r="55" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="10" t="s">
         <v>120</v>
       </c>
@@ -6007,7 +6024,7 @@
       <c r="K55" s="10"/>
       <c r="L55" s="10"/>
     </row>
-    <row r="56" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="10" t="s">
         <v>120</v>
       </c>
@@ -6037,7 +6054,7 @@
       <c r="K56" s="10"/>
       <c r="L56" s="10"/>
     </row>
-    <row r="57" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="10" t="s">
         <v>120</v>
       </c>
@@ -6067,7 +6084,7 @@
       <c r="K57" s="10"/>
       <c r="L57" s="10"/>
     </row>
-    <row r="58" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="10" t="s">
         <v>120</v>
       </c>
@@ -6097,7 +6114,7 @@
       <c r="K58" s="10"/>
       <c r="L58" s="10"/>
     </row>
-    <row r="59" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="10" t="s">
         <v>120</v>
       </c>
@@ -6127,7 +6144,7 @@
       <c r="K59" s="10"/>
       <c r="L59" s="10"/>
     </row>
-    <row r="60" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="10" t="s">
         <v>120</v>
       </c>
@@ -6157,7 +6174,7 @@
       <c r="K60" s="10"/>
       <c r="L60" s="10"/>
     </row>
-    <row r="61" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="10" t="s">
         <v>120</v>
       </c>
@@ -6187,7 +6204,7 @@
       <c r="K61" s="10"/>
       <c r="L61" s="10"/>
     </row>
-    <row r="62" spans="1:12" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:13" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="10" t="s">
         <v>120</v>
       </c>
@@ -6217,7 +6234,7 @@
       <c r="K62" s="10"/>
       <c r="L62" s="10"/>
     </row>
-    <row r="63" spans="1:12" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:13" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="10" t="s">
         <v>120</v>
       </c>
@@ -6231,10 +6248,10 @@
         <v>187</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>52</v>
+        <v>111</v>
       </c>
       <c r="F63" s="10" t="s">
-        <v>131</v>
+        <v>17</v>
       </c>
       <c r="G63" s="10" t="s">
         <v>18</v>
@@ -6246,8 +6263,11 @@
       <c r="J63" s="10"/>
       <c r="K63" s="10"/>
       <c r="L63" s="10"/>
-    </row>
-    <row r="64" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M63" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="10" t="s">
         <v>120</v>
       </c>
@@ -6277,7 +6297,7 @@
       <c r="K64" s="10"/>
       <c r="L64" s="10"/>
     </row>
-    <row r="65" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="10" t="s">
         <v>120</v>
       </c>
@@ -6294,7 +6314,7 @@
         <v>194</v>
       </c>
       <c r="F65" s="10" t="s">
-        <v>131</v>
+        <v>17</v>
       </c>
       <c r="G65" s="10" t="s">
         <v>18</v>
@@ -6306,8 +6326,11 @@
       <c r="J65" s="10"/>
       <c r="K65" s="10"/>
       <c r="L65" s="10"/>
-    </row>
-    <row r="66" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M65" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10" t="s">
         <v>195</v>
       </c>
@@ -6337,7 +6360,7 @@
       <c r="K66" s="10"/>
       <c r="L66" s="10"/>
     </row>
-    <row r="67" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="10" t="s">
         <v>195</v>
       </c>
@@ -6367,7 +6390,7 @@
       <c r="K67" s="10"/>
       <c r="L67" s="10"/>
     </row>
-    <row r="68" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="10" t="s">
         <v>195</v>
       </c>
@@ -6397,7 +6420,7 @@
       <c r="K68" s="10"/>
       <c r="L68" s="10"/>
     </row>
-    <row r="69" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="10" t="s">
         <v>195</v>
       </c>
@@ -6427,7 +6450,7 @@
       <c r="K69" s="10"/>
       <c r="L69" s="10"/>
     </row>
-    <row r="70" spans="1:12" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:13" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="10" t="s">
         <v>195</v>
       </c>
@@ -6457,7 +6480,7 @@
       <c r="K70" s="10"/>
       <c r="L70" s="10"/>
     </row>
-    <row r="71" spans="1:12" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:13" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="10" t="s">
         <v>195</v>
       </c>
@@ -6487,7 +6510,7 @@
       <c r="K71" s="18"/>
       <c r="L71" s="18"/>
     </row>
-    <row r="72" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="10" t="s">
         <v>195</v>
       </c>
@@ -6517,7 +6540,7 @@
       <c r="K72" s="10"/>
       <c r="L72" s="10"/>
     </row>
-    <row r="73" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="10" t="s">
         <v>195</v>
       </c>
@@ -6547,7 +6570,7 @@
       <c r="K73" s="10"/>
       <c r="L73" s="10"/>
     </row>
-    <row r="74" spans="1:12" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:13" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="10" t="s">
         <v>195</v>
       </c>
@@ -6577,7 +6600,7 @@
       <c r="K74" s="10"/>
       <c r="L74" s="10"/>
     </row>
-    <row r="75" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="10" t="s">
         <v>195</v>
       </c>
@@ -6607,7 +6630,7 @@
       <c r="K75" s="10"/>
       <c r="L75" s="10"/>
     </row>
-    <row r="76" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="10" t="s">
         <v>195</v>
       </c>
@@ -6637,7 +6660,7 @@
       <c r="K76" s="10"/>
       <c r="L76" s="10"/>
     </row>
-    <row r="77" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="10" t="s">
         <v>195</v>
       </c>
@@ -6667,7 +6690,7 @@
       <c r="K77" s="10"/>
       <c r="L77" s="10"/>
     </row>
-    <row r="78" spans="1:12" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:13" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="10" t="s">
         <v>195</v>
       </c>
@@ -6697,7 +6720,7 @@
       <c r="K78" s="10"/>
       <c r="L78" s="10"/>
     </row>
-    <row r="79" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="10" t="s">
         <v>195</v>
       </c>
@@ -6727,7 +6750,7 @@
       <c r="K79" s="10"/>
       <c r="L79" s="10"/>
     </row>
-    <row r="80" spans="1:12" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:13" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="10" t="s">
         <v>195</v>
       </c>
@@ -7976,11 +7999,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCFD84B1-2827-431B-9BB6-3A4D7786E114}">
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="27.85546875" customWidth="1"/>
     <col min="9" max="9" width="30.7109375" customWidth="1"/>
+    <col min="10" max="10" width="36.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8867,7 +8891,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="240" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" ht="240" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>298</v>
       </c>
@@ -8899,7 +8923,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="150" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" ht="150" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>298</v>
       </c>
@@ -8931,7 +8955,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="165" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" ht="165" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>298</v>
       </c>
@@ -8963,7 +8987,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="150" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" ht="150" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>298</v>
       </c>
@@ -8995,7 +9019,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>298</v>
       </c>
@@ -9018,7 +9042,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>298</v>
       </c>
@@ -9041,7 +9065,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>298</v>
       </c>
@@ -9064,7 +9088,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="210" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" ht="210" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>298</v>
       </c>
@@ -9096,7 +9120,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>298</v>
       </c>
@@ -9119,7 +9143,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>298</v>
       </c>
@@ -9142,7 +9166,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>298</v>
       </c>
@@ -9165,7 +9189,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>298</v>
       </c>
@@ -9188,7 +9212,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>298</v>
       </c>
@@ -9210,6 +9234,38 @@
       <c r="G45" s="2" t="s">
         <v>19</v>
       </c>
+    </row>
+    <row r="46" spans="1:12" ht="186" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B46" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="D46" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="E46" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G46" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="I46" s="10"/>
+      <c r="J46" s="10" t="s">
+        <v>713</v>
+      </c>
+      <c r="K46" s="10"/>
+      <c r="L46" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12256,26 +12312,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="139fca70-673f-44e1-94c2-b523bb9c108c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="7eaf932d-7370-48c5-9459-ae540daf9d7d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DFB9E5947890A84F90C1025035B3A9E9" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="abb99fc9a48c7a251434465201697796">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="139fca70-673f-44e1-94c2-b523bb9c108c" xmlns:ns3="7eaf932d-7370-48c5-9459-ae540daf9d7d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d5c101f0e739d89bf88b83005715ab8d" ns2:_="" ns3:_="">
     <xsd:import namespace="139fca70-673f-44e1-94c2-b523bb9c108c"/>
@@ -12482,32 +12518,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3BB2BB8B-BA4E-4835-AC34-431A62162A7D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="139fca70-673f-44e1-94c2-b523bb9c108c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="7eaf932d-7370-48c5-9459-ae540daf9d7d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B57CF69-5D19-450C-935B-68EC43A8DA31}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="139fca70-673f-44e1-94c2-b523bb9c108c"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="7eaf932d-7370-48c5-9459-ae540daf9d7d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82D5B6C7-9BF1-46B8-8CAF-B305B78CEC57}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12524,4 +12555,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B57CF69-5D19-450C-935B-68EC43A8DA31}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="139fca70-673f-44e1-94c2-b523bb9c108c"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="7eaf932d-7370-48c5-9459-ae540daf9d7d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3BB2BB8B-BA4E-4835-AC34-431A62162A7D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>